<commit_message>
Add 03/10 to 03/19 Sales Order Data
</commit_message>
<xml_diff>
--- a/Store Max Items.xlsx
+++ b/Store Max Items.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Desktop\inventoryprediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{407D0607-C775-4F19-9E84-BFBECFE565B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95190AEC-0FA7-4F6A-906A-8BFEF928E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F7753A57-749A-43F5-B214-517651157AC9}"/>
+    <workbookView xWindow="-23565" yWindow="0" windowWidth="21600" windowHeight="11385" xr2:uid="{F7753A57-749A-43F5-B214-517651157AC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -736,6 +736,7 @@
   <cols>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>